<commit_message>
개발안 Update(261002) 반영 — 1차
· Summary 장을 걷는다. 뒤의 세 장과 중복이라 둘 자리가 없다. 보고 이미지는 그 장을 통째로
  찍고 있었으므로, 이제 1·2·3을 직접 펼쳐 한 장으로 찍는다(차트가 '활성'일 때만 그려지므로
  찍기 전에 세 장을 한 번씩 열어 그려 둔다).

· 법인 행의 묶음과 차례를 새로 정한다 — HUK(HDG포함) · HUS · HJP · HUG · HSZ · HBR · 기타.
  기타는 HMX·HTR·HID·HAU다. 서버와 화면이 함께 보는 값이라 lib/corpGroups.ts로 떼어 두었고
  (aggregate를 그대로 들여오면 Supabase 서버 클라이언트가 브라우저 번들에 딸려 온다),
  배부판을 만들 때 한 번만 묶어 Summary 상세·App1·App3가 같은 차례를 쓴다.

· 누계 표 우측의 '1월~8월'을 뗀다. 표 제목이 이미 '8월 누계 실적'이라 같은 말이다. 단위(백만원)만
  남겼다 — 당월 표와 맞추고 단위 표기는 있어야 한다. EVCS 도넛 머리의 '누계 실적 기준'도 같은
  이유로 뗐다(왼쪽 표를 보면 안다).

· 코멘트: 법인 초과 문구를 'HBR tax credit 매각 수수료 650백만, Ciro 성공보수 54백만'으로 바꾸고
  상세 > 공통의 HBR 줄에도 같은 표현을 쓴다. 예산 초과·미집행 항목을 표와 같은 차례
  (STB > Mobility > EVCS > Humax(공통) > 건물)로 돌려 1~8월 전 구간에 적용했다.
  'Charter Legal fee/B&M Legal fee'의 뒤쪽 중복을 떼고, 합병 자문·평가 수수료에 법무법인 광장
  1월 10백만·4월 15백만을 더해 누계 482 → 506백만으로 고쳤다(8월분 8.8백만은 이미 들어 있었다).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Summary 작성용.xlsx
+++ b/Summary 작성용.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hyju\Desktop\클로드_고정비\fc-dashboard-web\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E854B20F-41FC-459F-981A-7FCC1AE0C086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1972058-882B-4E34-AEC0-1C8B5F653C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2550" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{C29230AE-43B5-4988-AB7A-BDE8403DF9F7}"/>
+    <workbookView xWindow="28680" yWindow="-885" windowWidth="29040" windowHeight="15720" xr2:uid="{C29230AE-43B5-4988-AB7A-BDE8403DF9F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -374,12 +374,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[지급수수료]
-New Aura/iWedia 외주개발용역비 518백만 추가 집행 가능성 있음 (SW이슈로 지연)
-Charter Legal fee/B&amp;M Legal fee 127백만 집행 (소송 재개)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1Q 월평균 278백만 → 2Q 월평균 126백만 (4월 한화 임대차 계약 영향)
 10월 사옥 이전 전까지 아래 비용 구조로 예상
@@ -437,20 +431,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>예산 대비 실적 집행률: 합계 2,976백만(120%), 본사 1,825백만(95%), 법인 1,152백만(204%)
- - 법인 초과: HBR 지급수수료 703백만 집행 — HBR Artur 세액공제 매각 중개수수료 650백만, HBR CTJ 법정 대표자 보수 54백만</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[인건비]
-주식보상비용 250백만 집행 (예산 외, 일회성)
-[지급수수료]
-8월 HBR 703백만 집행 (HBR Artur 세액공제 매각 중개수수료 650백만, HBR CTJ 법정 대표자 보수 54백만)
-합병 자문·평가 수수료 누계 482백만 집행 (7월 350백만, 8월 131백만)
-특허처리비 104백만 초과 집행 (VVC 예산 누락 영향)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>계단식 감소: 1Q 월평균 278백만 → 2Q 월평균 126백만 → 7월 154백만 → 8월 152백만
  - 4월~: 분당 감가상각비 163백만 → 분당 임차료 월 45백만
  - 7월~: 티맥스수내타워 임대차 관리비 29백만(총 58백만) 신규 반영</t>
@@ -513,12 +493,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>- 누계 실적 8,043백만(집행률 95%) — 예산 내 집행
-- 본사 5,646백만(집행률 90%) 예산 대비 미집행 · 법인 2,397백만(집행률 110%) 초과 — 방향 엇갈림
-- 항목별 집행률: 예산 초과 HUMAX(공통) 116%, MOBILITY 143% / 예산 미집행 STB 72%, 건물 94%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>- 누계 실적 1,417백만(집행률 72%) — 예산 대비 541백만 미집행
 - 예산 대비 Media그룹 -522백만(외주개발용역비 -533) 주원인 · 월 배부액 493→483→441백만 완만한 감소</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -530,12 +504,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>- 누계 실적 10,568백만(집행률 95%) — 예산 내 집행
-- 본사 7,514백만(집행률 91%) 예산 대비 미집행 · 법인 3,055백만(집행률 109%) 초과 — 방향 엇갈림
-- 항목별 집행률: 예산 초과 HUMAX(공통) 115%, EVCS(국내) 107% / 예산 미집행 건물 81%, STB 83%, EVCS(해외) 92%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>- 누계 실적 1,982백만(집행률 83%) — 예산 대비 410백만 미집행
 - 예산 대비 Media그룹 -426백만(외주개발용역비 -533) 주원인 · HUK +79백만 초과
 - 4월 트렌드 왜곡: STB License Fee/Nagra 4월 -84백만 (선급비용 결산 조정 지연)</t>
@@ -548,12 +516,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>- 누계 실적 13,012백만(집행률 97%) — 예산 내 집행
-- 본사 9,318백만(집행률 93%) 예산 대비 미집행 · 법인 3,694백만(집행률 108%) 초과 — 방향 엇갈림
-- 항목별 집행률: 예산 초과 HUMAX(공통) 121%, EVCS(국내) 110% / 예산 미집행 건물 72%, STB 85%, EVCS(해외) 92%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>- 누계 실적 2,381백만(집행률 85%) — 예산 대비 425백만 미집행
 - 예산 대비 Media그룹 -469백만(외주개발용역비 -525) 주원인 · 보정 후 월 441~493백만 — 감소 추세 없음
 - 4월, 5월 트렌드 왜곡: STB License Fee/Nagra 4월 -84백만, 5월 +84백만 (선급비용 결산 조정 지연)</t>
@@ -563,30 +525,6 @@
     <t>- 누계 실적 1,089백만(집행률 72%) — 예산 대비 416백만 미집행
 - 예산 대비 감가상각비 -326백만, 수도광열비 -168 미집행 주원인(임차료 +91 초과)
 - 1~3월 평균 278백만 → 4~5월 평균 128백만 — 4월부터 계단식 감소</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예산 대비 실적 집행률: 합계 15,549백만(97%), 본사 11,065백만(92%), 법인 4,484백만(112%)
- - 예산 초과: HUMAX(공통) 119%(주식보상 비용, VVC특허처리비 등) EVCS(국내) 108%
- - 예산 미집행: 건물 67%(1Q 94%, 2Q 41%), STB 90%, EVCS(해외) 94%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예산 대비 실적 집행률: 합계 18,210백만(98%), 본사 13,097백만(94%), 법인 5,112백만(111%)
- - 예산 초과: HUMAX(공통) 127%(합병 자문·평가 수수료, 주식보상 비용, VVC특허처리비 등) EVCS(국내) 108%
- - 예산 미집행: 건물 64%(1Q 94%, 2Q 41%, 7월 50%), STB 94%, EVCS(해외) 91%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예산 대비 실적 집행률: 합계 21,186백만(100%), 본사 14,922백만(94%), 법인 6,264백만(121%)
- - 예산 초과: HUMAX(공통) 141%(HBR 지급수수료, 합병 자문·평가 수수료 등) EVCS(국내) 108%
- - 예산 미집행: 건물 63%(1Q 94%, 2Q 41%, 3Q(7~8월) 51%), STB 95%, EVCS(해외) 90%</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[지급수수료]
-외주개발용역비 누계 229백만(집행률 30%) — 예산 대비 523백만 미집행 (New Aura/iWedia SW이슈로 지연)
-Charter Legal fee/B&amp;M Legal fee 8월 79백만 추가 집행 (누계 206백만, 소송 재개)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -607,6 +545,68 @@
     <t>1Q 월평균 278백만 → 2Q 월평균 126백만 → 7월 154백만 → 8월 152백만
  - 4월: 한화 임대차계약 체결로 구조 변경
  - 7월: 티맥스수내타워 관리비 집행 시작 · 8월 동일 구조 유지</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 누계 실적 8,043백만(집행률 95%) — 예산 내 집행
+- 본사 5,646백만(집행률 90%) 예산 대비 미집행 · 법인 2,397백만(집행률 110%) 초과 — 방향 엇갈림
+- 항목별 집행률: 예산 초과 MOBILITY 143%, HUMAX(공통) 116% / 예산 미집행 STB 72%, 건물 94%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 누계 실적 10,568백만(집행률 95%) — 예산 내 집행
+- 본사 7,514백만(집행률 91%) 예산 대비 미집행 · 법인 3,055백만(집행률 109%) 초과 — 방향 엇갈림
+- 항목별 집행률: 예산 초과 EVCS(국내) 107%, HUMAX(공통) 115% / 예산 미집행 STB 83%, EVCS(해외) 92%, 건물 81%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>- 누계 실적 13,012백만(집행률 97%) — 예산 내 집행
+- 본사 9,318백만(집행률 93%) 예산 대비 미집행 · 법인 3,694백만(집행률 108%) 초과 — 방향 엇갈림
+- 항목별 집행률: 예산 초과 EVCS(국내) 110%, HUMAX(공통) 121% / 예산 미집행 STB 85%, EVCS(해외) 92%, 건물 72%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예산 대비 실적 집행률: 합계 15,549백만(97%), 본사 11,065백만(92%), 법인 4,484백만(112%)
+ - 예산 초과: EVCS(국내) 108%, HUMAX(공통) 119%(주식보상 비용, VVC특허처리비 등)
+ - 예산 미집행: STB 90%, EVCS(해외) 94%, 건물 67%(1Q 94%, 2Q 41%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예산 대비 실적 집행률: 합계 18,210백만(98%), 본사 13,097백만(94%), 법인 5,112백만(111%)
+ - 예산 초과: EVCS(국내) 108%, HUMAX(공통) 127%(합병 자문·평가 수수료, 주식보상 비용, VVC특허처리비 등)
+ - 예산 미집행: STB 94%, EVCS(해외) 91%, 건물 64%(1Q 94%, 2Q 41%, 7월 50%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[지급수수료]
+New Aura/iWedia 외주개발용역비 518백만 추가 집행 가능성 있음 (SW이슈로 지연)
+Charter Legal fee/B&amp;M 127백만 집행 (소송 재개)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예산 대비 실적 집행률: 합계 2,976백만(120%), 본사 1,825백만(95%), 법인 1,152백만(204%)
+ - 법인 초과: HBR tax credit 매각 수수료 650백만, Ciro 성공보수 54백만</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예산 대비 실적 집행률: 합계 21,186백만(100%), 본사 14,922백만(94%), 법인 6,264백만(121%)
+ - 예산 초과: EVCS(국내) 108%, HUMAX(공통) 141%(HBR 지급수수료, 합병 자문·평가 수수료 등)
+ - 예산 미집행: STB 95%, EVCS(해외) 90%, 건물 63%(1Q 94%, 2Q 41%, 3Q(7~8월) 51%)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[지급수수료]
+외주개발용역비 누계 229백만(집행률 30%) — 예산 대비 523백만 미집행 (New Aura/iWedia SW이슈로 지연)
+Charter Legal fee/B&amp;M 8월 79백만 추가 집행 (누계 206백만, 소송 재개)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[인건비]
+주식보상비용 250백만 집행 (예산 외, 일회성)
+[지급수수료]
+8월 HBR 703백만 집행 (tax credit 매각 수수료 650백만, Ciro 성공보수 54백만)
+합병 자문·평가 수수료 누계 506백만 집행 (1월 10백만, 4월 15백만, 7월 350백만, 8월 131백만)
+특허처리비 104백만 초과 집행 (VVC 예산 누락 영향)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="49.5">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="49.5">
@@ -2375,7 +2375,7 @@
         <v>7</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="49.5">
@@ -2403,7 +2403,7 @@
         <v>9</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="49.5">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="49.5">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="49.5">
@@ -2453,7 +2453,7 @@
         <v>7</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="49.5">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="6" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="49.5">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="6" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="49.5">
@@ -2531,7 +2531,7 @@
         <v>7</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="49.5">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="49.5">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="7" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="49.5">
@@ -2609,7 +2609,7 @@
         <v>7</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="49.5">
@@ -2637,7 +2637,7 @@
         <v>9</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="49.5">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="49.5">
@@ -2687,7 +2687,7 @@
         <v>7</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="49.5">
@@ -2715,7 +2715,7 @@
         <v>9</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2808,10 +2808,10 @@
         <v>9</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="33">
@@ -2938,7 +2938,7 @@
         <v>7</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="E45" s="13" t="s">
         <v>58</v>
@@ -2955,7 +2955,7 @@
         <v>8</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E46" s="13" t="s">
         <v>58</v>
@@ -2972,7 +2972,7 @@
         <v>9</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E47" s="13" t="s">
         <v>59</v>
@@ -3023,7 +3023,7 @@
         <v>9</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E50" s="13" t="s">
         <v>60</v>
@@ -3034,11 +3034,11 @@
         <v>4</v>
       </c>
       <c r="B51" s="25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C51" s="25"/>
       <c r="D51" s="8" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="E51" s="24" t="s">
         <v>54</v>
@@ -3049,11 +3049,11 @@
         <v>4</v>
       </c>
       <c r="B52" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C52" s="25"/>
       <c r="D52" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E52" s="24" t="s">
         <v>54</v>
@@ -3064,11 +3064,11 @@
         <v>5</v>
       </c>
       <c r="B53" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C53" s="25"/>
       <c r="D53" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E53" s="24" t="s">
         <v>57</v>
@@ -3079,13 +3079,13 @@
         <v>6</v>
       </c>
       <c r="B54" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C54" s="25" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E54" s="24" t="s">
         <v>58</v>
@@ -3096,13 +3096,13 @@
         <v>6</v>
       </c>
       <c r="B55" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C55" s="25" t="s">
         <v>8</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="E55" s="24" t="s">
         <v>58</v>
@@ -3113,13 +3113,13 @@
         <v>6</v>
       </c>
       <c r="B56" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C56" s="25" t="s">
         <v>9</v>
       </c>
       <c r="D56" s="26" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="E56" s="24" t="s">
         <v>59</v>
@@ -3130,13 +3130,13 @@
         <v>44</v>
       </c>
       <c r="B57" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C57" s="25" t="s">
         <v>7</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E57" s="24" t="s">
         <v>60</v>
@@ -3147,13 +3147,13 @@
         <v>44</v>
       </c>
       <c r="B58" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C58" s="25" t="s">
         <v>8</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E58" s="24" t="s">
         <v>60</v>
@@ -3164,13 +3164,13 @@
         <v>44</v>
       </c>
       <c r="B59" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C59" s="25" t="s">
         <v>9</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E59" s="24" t="s">
         <v>60</v>
@@ -3266,7 +3266,7 @@
     <row r="82" spans="1:4">
       <c r="A82" s="27"/>
       <c r="D82" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>